<commit_message>
Fix voter import constraint errors, ElectionSetup Step 4 icon reference, and update master spreadsheets
</commit_message>
<xml_diff>
--- a/Smart EVM - Candidates for All Constituencies.xlsx
+++ b/Smart EVM - Candidates for All Constituencies.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -563,11 +563,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="F2" s="3" t="inlineStr"/>
       <c r="G2" s="3" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -576,12 +574,12 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>TDP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Telugu Desam Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -607,11 +605,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F3" s="5" t="n">
-        <v>5</v>
-      </c>
+      <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
@@ -620,12 +616,12 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -651,11 +647,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F4" s="3" t="inlineStr"/>
       <c r="G4" s="3" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -664,12 +658,12 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -697,7 +691,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
@@ -737,11 +731,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F6" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -750,12 +742,12 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -781,11 +773,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n">
-        <v>7</v>
-      </c>
+      <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -794,12 +784,12 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>BJP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Bharatiya Janata Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -825,11 +815,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -838,12 +826,12 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -871,7 +859,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -911,11 +899,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -924,12 +910,12 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -955,11 +941,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="5" t="n">
-        <v>4</v>
-      </c>
+      <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -968,12 +952,12 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>TDP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Telugu Desam Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -999,11 +983,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F12" s="3" t="inlineStr"/>
       <c r="G12" s="3" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -1012,12 +994,12 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1027,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -1085,12 +1067,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G14" s="3" t="n">
-        <v>25</v>
-      </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Proddatur</t>
@@ -1098,12 +1078,12 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>TDP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Telugu Desam Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1129,11 +1109,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F15" s="5" t="n">
-        <v>5</v>
-      </c>
+      <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -1142,12 +1120,12 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1173,11 +1151,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F16" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F16" s="3" t="inlineStr"/>
       <c r="G16" s="3" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1186,12 +1162,12 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1195,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr"/>
       <c r="G17" s="5" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -1259,11 +1235,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F18" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="F18" s="3" t="inlineStr"/>
       <c r="G18" s="3" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1272,12 +1246,12 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>TDP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Telugu Desam Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1303,12 +1277,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F19" s="5" t="n">
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G19" s="5" t="n">
-        <v>26</v>
-      </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Kurnool</t>
@@ -1316,12 +1288,12 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1347,11 +1319,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F20" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F20" s="3" t="inlineStr"/>
       <c r="G20" s="3" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1360,12 +1330,12 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1363,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
@@ -1433,11 +1403,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F22" s="3" t="n">
-        <v>7</v>
-      </c>
+      <c r="F22" s="3" t="inlineStr"/>
       <c r="G22" s="3" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -1446,12 +1414,12 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>BJP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Bharatiya Janata Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1477,11 +1445,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F23" s="5" t="n">
-        <v>5</v>
-      </c>
+      <c r="F23" s="5" t="inlineStr"/>
       <c r="G23" s="5" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
@@ -1490,12 +1456,12 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1521,11 +1487,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F24" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F24" s="3" t="inlineStr"/>
       <c r="G24" s="3" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -1534,12 +1498,12 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1531,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr"/>
       <c r="G25" s="5" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
@@ -1607,11 +1571,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F26" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="F26" s="3" t="inlineStr"/>
       <c r="G26" s="3" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -1620,12 +1582,12 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>TDP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Telugu Desam Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1651,11 +1613,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F27" s="5" t="n">
-        <v>5</v>
-      </c>
+      <c r="F27" s="5" t="inlineStr"/>
       <c r="G27" s="5" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
@@ -1664,12 +1624,12 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1695,11 +1655,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F28" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F28" s="3" t="inlineStr"/>
       <c r="G28" s="3" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1708,12 +1666,12 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1699,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="5" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
@@ -1781,11 +1739,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F30" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="F30" s="3" t="inlineStr"/>
       <c r="G30" s="3" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1794,12 +1750,12 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>TDP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Telugu Desam Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1825,11 +1781,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F31" s="5" t="n">
-        <v>5</v>
-      </c>
+      <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="5" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
@@ -1838,12 +1792,12 @@
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1869,12 +1823,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F32" s="3" t="n">
+      <c r="F32" s="3" t="inlineStr"/>
+      <c r="G32" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="G32" s="3" t="n">
-        <v>29</v>
-      </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Nandyal</t>
@@ -1882,12 +1834,12 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1867,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr"/>
       <c r="G33" s="5" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
@@ -1955,11 +1907,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F34" s="3" t="n">
-        <v>6</v>
-      </c>
+      <c r="F34" s="3" t="inlineStr"/>
       <c r="G34" s="3" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -1968,12 +1918,12 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>JSP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Jana Sena Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -1999,11 +1949,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F35" s="5" t="n">
-        <v>5</v>
-      </c>
+      <c r="F35" s="5" t="inlineStr"/>
       <c r="G35" s="5" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
@@ -2012,12 +1960,12 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2043,11 +1991,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F36" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F36" s="3" t="inlineStr"/>
       <c r="G36" s="3" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -2056,12 +2002,12 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2035,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr"/>
       <c r="G37" s="5" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
@@ -2129,11 +2075,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F38" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="F38" s="3" t="inlineStr"/>
       <c r="G38" s="3" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -2142,12 +2086,12 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>TDP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Telugu Desam Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2173,11 +2117,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F39" s="5" t="n">
-        <v>5</v>
-      </c>
+      <c r="F39" s="5" t="inlineStr"/>
       <c r="G39" s="5" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
@@ -2186,12 +2128,12 @@
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2217,11 +2159,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F40" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F40" s="3" t="inlineStr"/>
       <c r="G40" s="3" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -2230,12 +2170,12 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2203,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr"/>
       <c r="G41" s="5" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
@@ -2303,11 +2243,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F42" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="F42" s="3" t="inlineStr"/>
       <c r="G42" s="3" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
@@ -2316,12 +2254,12 @@
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>TDP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Telugu Desam Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2347,11 +2285,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F43" s="5" t="n">
-        <v>5</v>
-      </c>
+      <c r="F43" s="5" t="inlineStr"/>
       <c r="G43" s="5" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
@@ -2360,12 +2296,12 @@
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2391,11 +2327,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F44" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F44" s="3" t="inlineStr"/>
       <c r="G44" s="3" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -2404,12 +2338,12 @@
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2371,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr"/>
       <c r="G45" s="5" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
@@ -2477,11 +2411,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F46" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="F46" s="3" t="inlineStr"/>
       <c r="G46" s="3" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2490,12 +2422,12 @@
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>TDP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Telugu Desam Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2521,11 +2453,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F47" s="5" t="n">
-        <v>5</v>
-      </c>
+      <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="5" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
@@ -2534,12 +2464,12 @@
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>YSRCP</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
         <is>
-          <t>YSR Congress Party</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2565,11 +2495,9 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F48" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="F48" s="3" t="inlineStr"/>
       <c r="G48" s="3" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2578,12 +2506,12 @@
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>INC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Independent</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2539,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr"/>
       <c r="G49" s="5" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="H49" s="4" t="inlineStr">
         <is>
@@ -2624,180 +2552,6 @@
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Praveen Khandelwal</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="n">
-        <v>63</v>
-      </c>
-      <c r="C50" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>LL.B</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="G50" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>Central Delhi</t>
-        </is>
-      </c>
-      <c r="I50" s="3" t="inlineStr">
-        <is>
-          <t>BJP</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>Bharatiya Janata Party</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>Jai Prakash Agarwal</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="n">
-        <v>78</v>
-      </c>
-      <c r="C51" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>B.A.</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="G51" s="5" t="n">
-        <v>34</v>
-      </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>Central Delhi</t>
-        </is>
-      </c>
-      <c r="I51" s="5" t="inlineStr">
-        <is>
-          <t>INC</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
-        <is>
-          <t>Indian National Congress</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Somnath Bharti</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="C52" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>M.Sc, LL.B</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="G52" s="3" t="n">
-        <v>34</v>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>Central Delhi</t>
-        </is>
-      </c>
-      <c r="I52" s="3" t="inlineStr">
-        <is>
-          <t>AAP</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>Aam Aadmi Party</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>Rajiv Sharma</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="C53" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>B.Tech</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F53" s="5" t="inlineStr"/>
-      <c r="G53" s="5" t="n">
-        <v>34</v>
-      </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>Central Delhi</t>
-        </is>
-      </c>
-      <c r="I53" s="5" t="inlineStr">
-        <is>
-          <t>IND</t>
-        </is>
-      </c>
-      <c r="J53" s="4" t="inlineStr">
         <is>
           <t>Independent</t>
         </is>
@@ -2814,7 +2568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2867,7 +2621,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -2880,28 +2634,14 @@
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>TDP</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Telugu Desam Party</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Bicycle</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -2914,28 +2654,14 @@
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>YSRCP</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>YSR Congress Party</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Ceiling Fan</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -2948,28 +2674,14 @@
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>JSP</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Jana Sena Party</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Glass Tumbler</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -2982,28 +2694,14 @@
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="n">
-        <v>7</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>BJP</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Bharatiya Janata Party</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Lotus</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -3016,28 +2714,14 @@
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>INC</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Indian National Congress</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Hand</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -3050,28 +2734,14 @@
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="n">
-        <v>9</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>AAP</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Aam Aadmi Party</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Broom</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -3091,7 +2761,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -3111,7 +2781,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -3131,7 +2801,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -3151,7 +2821,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -3171,7 +2841,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -3189,26 +2859,6 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
     </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>34</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>DL-01</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Central Delhi</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>